<commit_message>
Knowledge base: one-click bridge enable + Chrome local-network hint
On the deployed https site the AI-brain Bridge setting defaults to
"Auto — probe on localhost only", so Settings → Knowledge base sat in its
"switched off" state and Re-check looked dead. The bridge-down panel now
offers "Enable the bridge on this device" (sets bridge:'on' per device and
re-checks) and, on https origins, explains Chrome's local-network permission
prompt, which otherwise stalls the probe silently. Workbook row A-033.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/App-audit-and-tasks.xlsx
+++ b/App-audit-and-tasks.xlsx
@@ -2940,20 +2940,76 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n"/>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="6" t="n"/>
-      <c r="H33" s="6" t="n"/>
-      <c r="I33" s="6" t="n"/>
-      <c r="J33" s="6" t="n"/>
-      <c r="K33" s="7" t="n"/>
-      <c r="L33" s="5" t="n"/>
-      <c r="M33" s="5" t="n"/>
-      <c r="N33" s="5" t="n"/>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>A-033</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>On the deployed site (https), Settings → Knowledge base → Re-check appeared to do nothing. Two causes found live on Ace's Mac 2026-09-08: (1) AI brain → Bridge defaults to 'Auto — probe on localhost only', so a deployed page never contacts the bridge and the section stays in its 'switched off' state; (2) Chrome 152 pauses a public-https → 127.0.0.1 fetch behind a local-network permission prompt, so the probe hangs until the user clicks Allow.</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Phase 4 - UX &amp; Accessibility</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Add a one-click 'Enable the bridge on this device' button and a Chrome local-network hint to the Knowledge base bridge-down state</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>src/services/knowledge.js (bridgeOff / enableBridgeHere / localNetworkNote); src/components/KnowledgeSection.jsx bridge-down panel; src/services/ai.js:93 bridgeEnabled() ('auto' = localhost only)</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>knowledge.js exports bridgeOff() (= !bridgeEnabled()), enableBridgeHere() (setAiSettings({ bridge:'on' }) then refreshKnowledge()) and localNetworkNote() (text shown only on https non-local origins). KnowledgeSection shows the button when the bridge is off and the note under the bridge-down panel. Per-device setting, same storage as the rest of the AI settings (task-monitor.ai-settings.v1).</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>A user on tasks.blueinnovation.ph can turn the bridge on from the Knowledge base section itself and is told to accept Chrome's local-network prompt; Re-check then reaches the bridge on their Mac.</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>Verified: lint clean, 49 tests pass, build clean. Live: after setting bridge:'on' in the browser the section moved from 'switched off' to 'Checking…' and probed 127.0.0.1:4319; the probe waits on Chrome's local-network permission until the user clicks Allow (cannot be clicked by automation).</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>A-026</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>XS (&lt;15m)</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>

</xml_diff>